<commit_message>
Incorporated review comments dated 20.04
</commit_message>
<xml_diff>
--- a/spice-auction-pwa/backend/data/SOURCE.xlsx
+++ b/spice-auction-pwa/backend/data/SOURCE.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4512" uniqueCount="2275">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4524" uniqueCount="2278">
   <si>
     <t>NAME</t>
   </si>
@@ -4105,7 +4105,7 @@
     <t>8838618302</t>
   </si>
   <si>
-    <t>11227657026</t>
+    <t>112276570262</t>
   </si>
   <si>
     <t>KALAIARASAN.M</t>
@@ -6836,6 +6836,15 @@
   </si>
   <si>
     <t>1234567890654</t>
+  </si>
+  <si>
+    <t>PRIYA</t>
+  </si>
+  <si>
+    <t>0987663728</t>
+  </si>
+  <si>
+    <t>10,salai</t>
   </si>
 </sst>
 </file>
@@ -7216,7 +7225,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L376"/>
+  <dimension ref="A1:L377"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -21520,6 +21529,44 @@
         <v>2274</v>
       </c>
     </row>
+    <row r="377" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A377" t="s">
+        <v>2275</v>
+      </c>
+      <c r="B377" t="s">
+        <v>2244</v>
+      </c>
+      <c r="C377" t="s">
+        <v>2245</v>
+      </c>
+      <c r="D377" t="s">
+        <v>2276</v>
+      </c>
+      <c r="E377" t="s">
+        <v>16</v>
+      </c>
+      <c r="F377" t="s">
+        <v>2277</v>
+      </c>
+      <c r="G377" t="s">
+        <v>2247</v>
+      </c>
+      <c r="H377" t="s">
+        <v>2248</v>
+      </c>
+      <c r="I377" t="s">
+        <v>1074</v>
+      </c>
+      <c r="J377" t="s">
+        <v>32</v>
+      </c>
+      <c r="K377" t="s">
+        <v>1680</v>
+      </c>
+      <c r="L377" t="s">
+        <v>1748</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>